<commit_message>
fix(kuya-marvin): tracker v2 - wrapped/full instruction text, who-writes-what legend, sample rows (yellow) in DailyLog+Earnings, one-row-per-day rule
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/clients/oceanides/kuya-marvin/tracker/kuya-marvin-tracker.xlsx
+++ b/clients/oceanides/kuya-marvin/tracker/kuya-marvin-tracker.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="48">
   <si>
     <t>KUYA MARVIN NG OCEANIDES</t>
   </si>
@@ -21,7 +21,7 @@
     <t>WEEKLY PAYSLIP — Attendance &amp; Earnings Tracker</t>
   </si>
   <si>
-    <t>Week start (Lunes)</t>
+    <t>Week start (Lunes) — si Neil ang nagpapalit kada Lunes</t>
   </si>
   <si>
     <t>Days worked</t>
@@ -39,22 +39,25 @@
     <t>TOTAL PAYOUT (kada Sabado, GCash)</t>
   </si>
   <si>
-    <t>PAANO GAMITIN:</t>
-  </si>
-  <si>
-    <t>1. Si Marvin ang nag-fi-fill ng DailyLog at Earnings — maliban sa column na "Bayad na?".</t>
-  </si>
-  <si>
-    <t>2. Ang "Bayad na?" (Earnings, col F) ay si Neil LANG: OO kapag nakolekta na ang bayad ng client.</t>
-  </si>
-  <si>
-    <t>3. Ang commission ay pumapasok sa payslip kapag OO na — hindi sa booking pa lang.</t>
-  </si>
-  <si>
-    <t>4. Kada Lunes, palitan ang "Week start" sa taas.</t>
-  </si>
-  <si>
-    <t>5. Commission: Certified = P250 | Lusong = 5% ng deal | Maintenance = P500 (auto na sa Earnings).</t>
+    <t>PAANO GAMITIN — SINO ANG NAGSUSULAT:</t>
+  </si>
+  <si>
+    <t>1.  Si MARVIN ang nagsusulat sa DailyLog (lahat ng columns) at sa Earnings columns A hanggang D — araw-araw.</t>
+  </si>
+  <si>
+    <t>2.  Si NEIL LANG ang nagsusulat sa "Bayad na?" (Earnings column F): OO kapag nakolekta na ang bayad ng client. Si Neil din ang nagpapalit ng Week start sa taas kada Lunes.</t>
+  </si>
+  <si>
+    <t>3.  DailyLog: ISANG row kada working day. Pagsamahin sa Notes kung maraming ginawa sa isang araw.</t>
+  </si>
+  <si>
+    <t>4.  Ang commission ay pumapasok sa payslip kapag OO na ang "Bayad na?" — hindi sa booking pa lang.</t>
+  </si>
+  <si>
+    <t>5.  Commission: Certified = P250  |  Lusong = 5% ng deal  |  Maintenance = P500. Auto-compute na ito sa Earnings — piliin lang ang Uri at ilagay ang halaga ng deal.</t>
+  </si>
+  <si>
+    <t>6.  May HALIMBAWA rows (dilaw na background) sa DailyLog at Earnings — tingnan para makita ang tamang pag-fill, tapos BURAHIN kapag magsisimula na ang totoong logging.</t>
   </si>
   <si>
     <t>Petsa</t>
@@ -75,10 +78,55 @@
     <t>Transport (P)</t>
   </si>
   <si>
-    <t>Notes</t>
-  </si>
-  <si>
-    <t>Client</t>
+    <t>Notes  (si Marvin ang nagsusulat sa tab na ito)</t>
+  </si>
+  <si>
+    <t>Inspection</t>
+  </si>
+  <si>
+    <t>Aling Rosa — Project 8, QC</t>
+  </si>
+  <si>
+    <t>8:30 AM</t>
+  </si>
+  <si>
+    <t>10:00 AM</t>
+  </si>
+  <si>
+    <t>HALIMBAWA: septic check, kuha photos, report sa group chat</t>
+  </si>
+  <si>
+    <t>Canvass</t>
+  </si>
+  <si>
+    <t>5 restaurants sa Maginhawa</t>
+  </si>
+  <si>
+    <t>1:00 PM</t>
+  </si>
+  <si>
+    <t>4:30 PM</t>
+  </si>
+  <si>
+    <t>HALIMBAWA: nag-iwan ng contact, 2 ang interesado sa Health Check</t>
+  </si>
+  <si>
+    <t>Content</t>
+  </si>
+  <si>
+    <t>Shoot — reference photos</t>
+  </si>
+  <si>
+    <t>9:00 AM</t>
+  </si>
+  <si>
+    <t>12:00 PM</t>
+  </si>
+  <si>
+    <t>HALIMBAWA: burahin ang mga dilaw na row kapag magsisimula na</t>
+  </si>
+  <si>
+    <t>Client  (si Marvin: A–D)</t>
   </si>
   <si>
     <t>Uri</t>
@@ -87,10 +135,28 @@
     <t>Halaga ng deal (P)</t>
   </si>
   <si>
-    <t>Commission (P)</t>
-  </si>
-  <si>
-    <t>Bayad na? (si Neil lang)</t>
+    <t>Commission (P) — AUTO</t>
+  </si>
+  <si>
+    <t>Bayad na? (si NEIL lang)</t>
+  </si>
+  <si>
+    <t>ABC Restaurant Corp. (5 loads, may DENR cert)</t>
+  </si>
+  <si>
+    <t>Certified</t>
+  </si>
+  <si>
+    <t>OO</t>
+  </si>
+  <si>
+    <t>Aling Rosa — lusong mula sa Health Check</t>
+  </si>
+  <si>
+    <t>Lusong</t>
+  </si>
+  <si>
+    <t>HINDI</t>
   </si>
 </sst>
 </file>
@@ -101,7 +167,7 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="&quot;₱&quot;#,##0"/>
   </numFmts>
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="12" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -158,8 +224,13 @@
       <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
+    <font>
+      <i/>
+      <color rgb="FF13293D"/>
+      <sz val="10.5"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -194,6 +265,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF5B301"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF7DF"/>
       </patternFill>
     </fill>
   </fills>
@@ -248,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -284,10 +360,10 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -300,6 +376,9 @@
     <xf numFmtId="165" fontId="10" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="165" fontId="11" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -647,12 +726,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
-    <col min="2" max="2" width="34" customWidth="1"/>
-    <col min="3" max="3" width="20" customWidth="1"/>
+    <col min="2" max="2" width="44" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="3" customWidth="1"/>
   </cols>
   <sheetData>
@@ -720,44 +799,50 @@
         <f>C7+C8+C9</f>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="13" ht="18" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B13" s="12" t="s">
         <v>8</v>
       </c>
       <c r="C13" s="12"/>
     </row>
-    <row r="14" ht="16" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="14" ht="30" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B14" s="13" t="s">
         <v>9</v>
       </c>
       <c r="C14" s="13"/>
     </row>
-    <row r="15" ht="16" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="15" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B15" s="13" t="s">
         <v>10</v>
       </c>
       <c r="C15" s="13"/>
     </row>
-    <row r="16" ht="16" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="16" ht="30" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B16" s="13" t="s">
         <v>11</v>
       </c>
       <c r="C16" s="13"/>
     </row>
-    <row r="17" ht="16" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="17" ht="30" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B17" s="13" t="s">
         <v>12</v>
       </c>
       <c r="C17" s="13"/>
     </row>
-    <row r="18" ht="16" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+    <row r="18" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B18" s="13" t="s">
         <v>13</v>
       </c>
       <c r="C18" s="13"/>
     </row>
+    <row r="19" ht="42" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B19" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="13"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B13:C13"/>
@@ -766,6 +851,7 @@
     <mergeCell ref="B16:C16"/>
     <mergeCell ref="B17:C17"/>
     <mergeCell ref="B18:C18"/>
+    <mergeCell ref="B19:C19"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -774,38 +860,105 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G1"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" style="14" customWidth="1"/>
     <col min="2" max="2" width="18" customWidth="1"/>
-    <col min="3" max="3" width="26" customWidth="1"/>
+    <col min="3" max="3" width="30" customWidth="1"/>
     <col min="4" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="13" style="15" customWidth="1"/>
-    <col min="7" max="7" width="40" customWidth="1"/>
+    <col min="7" max="7" width="52" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="D1" s="17" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E1" s="17" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F1" s="18" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G1" s="17" t="s">
-        <v>20</v>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" s="19">
+        <v>46223.66666666667</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="20" t="s">
+        <v>25</v>
+      </c>
+      <c r="F2" s="21">
+        <v>250</v>
+      </c>
+      <c r="G2" s="20" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="19">
+        <v>46224.66666666667</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="21">
+        <v>200</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="19">
+        <v>46225.66666666667</v>
+      </c>
+      <c r="B4" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C4" s="20" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" s="20" t="s">
+        <v>34</v>
+      </c>
+      <c r="E4" s="20" t="s">
+        <v>35</v>
+      </c>
+      <c r="F4" s="21"/>
+      <c r="G4" s="20" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -825,41 +978,71 @@
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="13" style="14" customWidth="1"/>
-    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="2" max="2" width="30" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="17" style="15" customWidth="1"/>
-    <col min="5" max="5" width="15" style="15" customWidth="1"/>
-    <col min="6" max="6" width="20" customWidth="1"/>
+    <col min="5" max="5" width="20" style="15" customWidth="1"/>
+    <col min="6" max="6" width="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="16" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="D1" s="18" t="s">
-        <v>23</v>
+        <v>39</v>
       </c>
       <c r="E1" s="18" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="F1" s="17" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="2" spans="5:5" x14ac:dyDescent="0.25">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="19">
+        <v>46223.66666666667</v>
+      </c>
+      <c r="B2" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="21">
+        <v>12000</v>
+      </c>
       <c r="E2" s="15">
         <f>IF($C2="Certified",250,IF($C2="Lusong",$D2*0.05,IF($C2="Maintenance",500,"")))</f>
       </c>
-    </row>
-    <row r="3" spans="5:5" x14ac:dyDescent="0.25">
+      <c r="F2" s="20" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="19">
+        <v>46225.66666666667</v>
+      </c>
+      <c r="B3" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="C3" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D3" s="21">
+        <v>20000</v>
+      </c>
       <c r="E3" s="15">
         <f>IF($C3="Certified",250,IF($C3="Lusong",$D3*0.05,IF($C3="Maintenance",500,"")))</f>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>47</v>
       </c>
     </row>
     <row r="4" spans="5:5" x14ac:dyDescent="0.25">

</xml_diff>